<commit_message>
Cập nhật báo cáo
</commit_message>
<xml_diff>
--- a/api/src/TAKAHATA.Api/Templates/detail_template.xlsx
+++ b/api/src/TAKAHATA.Api/Templates/detail_template.xlsx
@@ -13255,36 +13255,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="4" fontId="34" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -13337,6 +13307,36 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -14110,11 +14110,11 @@
         </c:ser>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="138521600"/>
-        <c:axId val="138535680"/>
+        <c:axId val="105451520"/>
+        <c:axId val="105453056"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="138521600"/>
+        <c:axId val="105451520"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -14152,14 +14152,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="138535680"/>
+        <c:crossAx val="105453056"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="138535680"/>
+        <c:axId val="105453056"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -14203,7 +14203,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="138521600"/>
+        <c:crossAx val="105451520"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -14296,7 +14296,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{042FA6C6-A9A6-B020-0B1E-06FF741790E1}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{042FA6C6-A9A6-B020-0B1E-06FF741790E1}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -14339,7 +14339,7 @@
         <xdr:cNvPr id="210843" name="Group 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E441A73F-6BDA-F1EC-8A02-B0FEF638374D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{E441A73F-6BDA-F1EC-8A02-B0FEF638374D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -14360,7 +14360,7 @@
           <xdr:cNvPr id="3" name="Rectangle 2">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EB311355-5A13-3CE4-04AD-EBD423245796}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{EB311355-5A13-3CE4-04AD-EBD423245796}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -14435,7 +14435,7 @@
           <xdr:cNvPr id="4" name="Rectangle 3">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1DDA0C9F-6125-69F0-C735-56A1D79E75C6}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{1DDA0C9F-6125-69F0-C735-56A1D79E75C6}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -14505,7 +14505,7 @@
           <xdr:cNvPr id="5" name="Rectangle 4">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{66DCDBC1-B5EE-4256-EE82-D65A8ADBF313}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{66DCDBC1-B5EE-4256-EE82-D65A8ADBF313}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -14591,7 +14591,7 @@
         <xdr:cNvPr id="6" name="Rectangle 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4891A1A4-CFC8-B7BC-616E-060F77A4F404}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{4891A1A4-CFC8-B7BC-616E-060F77A4F404}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -15117,12 +15117,14 @@
     <col min="2" max="2" width="16.42578125" style="244" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="10.42578125" style="264" customWidth="1"/>
     <col min="4" max="4" width="22.28515625" style="264" customWidth="1"/>
-    <col min="5" max="5" width="9" style="258" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" style="244" customWidth="1"/>
+    <col min="5" max="5" width="30.140625" style="258" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" style="244" customWidth="1"/>
     <col min="7" max="7" width="30.42578125" style="244" customWidth="1"/>
     <col min="8" max="9" width="12.5703125" style="244" customWidth="1"/>
     <col min="10" max="10" width="12.5703125" style="268" customWidth="1"/>
-    <col min="11" max="13" width="10.42578125" style="244" customWidth="1"/>
+    <col min="11" max="11" width="10.42578125" style="244" customWidth="1"/>
+    <col min="12" max="12" width="14.42578125" style="244" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" style="244" customWidth="1"/>
     <col min="14" max="14" width="14.7109375" style="244" customWidth="1"/>
     <col min="15" max="15" width="12" style="265" customWidth="1"/>
     <col min="16" max="16" width="15.7109375" style="265" customWidth="1"/>
@@ -15238,81 +15240,81 @@
       <c r="Q5" s="261"/>
     </row>
     <row r="6" spans="1:19" ht="26.25" customHeight="1" thickBot="1">
-      <c r="A6" s="273" t="s">
+      <c r="A6" s="291" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="281" t="s">
+      <c r="B6" s="299" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="277" t="s">
+      <c r="C6" s="295" t="s">
         <v>3627</v>
       </c>
-      <c r="D6" s="277" t="s">
+      <c r="D6" s="295" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="285" t="s">
+      <c r="E6" s="275" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="293" t="s">
+      <c r="F6" s="283" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="279" t="s">
+      <c r="G6" s="297" t="s">
         <v>1</v>
       </c>
-      <c r="H6" s="287" t="s">
+      <c r="H6" s="277" t="s">
         <v>4</v>
       </c>
-      <c r="I6" s="288"/>
-      <c r="J6" s="275" t="s">
+      <c r="I6" s="278"/>
+      <c r="J6" s="293" t="s">
         <v>3870</v>
       </c>
-      <c r="K6" s="297" t="s">
+      <c r="K6" s="287" t="s">
         <v>10</v>
       </c>
-      <c r="L6" s="298"/>
-      <c r="M6" s="299" t="s">
+      <c r="L6" s="288"/>
+      <c r="M6" s="289" t="s">
         <v>8</v>
       </c>
-      <c r="N6" s="295" t="s">
+      <c r="N6" s="285" t="s">
         <v>3</v>
       </c>
-      <c r="O6" s="292" t="s">
+      <c r="O6" s="282" t="s">
         <v>9</v>
       </c>
-      <c r="P6" s="283" t="s">
+      <c r="P6" s="273" t="s">
         <v>29</v>
       </c>
-      <c r="Q6" s="289" t="s">
+      <c r="Q6" s="279" t="s">
         <v>13</v>
       </c>
-      <c r="R6" s="290"/>
-      <c r="S6" s="291"/>
+      <c r="R6" s="280"/>
+      <c r="S6" s="281"/>
     </row>
     <row r="7" spans="1:19" ht="27.75" customHeight="1">
-      <c r="A7" s="274"/>
-      <c r="B7" s="282"/>
-      <c r="C7" s="278"/>
-      <c r="D7" s="278"/>
-      <c r="E7" s="286"/>
-      <c r="F7" s="294"/>
-      <c r="G7" s="280"/>
+      <c r="A7" s="292"/>
+      <c r="B7" s="300"/>
+      <c r="C7" s="296"/>
+      <c r="D7" s="296"/>
+      <c r="E7" s="276"/>
+      <c r="F7" s="284"/>
+      <c r="G7" s="298"/>
       <c r="H7" s="267" t="s">
         <v>3871</v>
       </c>
       <c r="I7" s="262" t="s">
         <v>2</v>
       </c>
-      <c r="J7" s="276"/>
+      <c r="J7" s="294"/>
       <c r="K7" s="263" t="s">
         <v>7</v>
       </c>
       <c r="L7" s="263" t="s">
         <v>3872</v>
       </c>
-      <c r="M7" s="300"/>
-      <c r="N7" s="296"/>
-      <c r="O7" s="284"/>
-      <c r="P7" s="284"/>
+      <c r="M7" s="290"/>
+      <c r="N7" s="286"/>
+      <c r="O7" s="274"/>
+      <c r="P7" s="274"/>
       <c r="Q7" s="271" t="s">
         <v>3867</v>
       </c>
@@ -15325,6 +15327,12 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="J6:J7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="D6:D7"/>
     <mergeCell ref="P6:P7"/>
     <mergeCell ref="E6:E7"/>
     <mergeCell ref="H6:I6"/>
@@ -15334,12 +15342,6 @@
     <mergeCell ref="N6:N7"/>
     <mergeCell ref="K6:L6"/>
     <mergeCell ref="M6:M7"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="J6:J7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="D6:D7"/>
   </mergeCells>
   <phoneticPr fontId="37" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.23622047244094499" bottom="0" header="0.31496062992126" footer="0.31496062992126"/>

</xml_diff>